<commit_message>
changes c60 to 0.1uF to fix oscillation problem, add GERBER.zip for Fab
</commit_message>
<xml_diff>
--- a/Smart Charger Files/Docs/BOMs/SC Rev B 250413 BOM 250501.xlsx
+++ b/Smart Charger Files/Docs/BOMs/SC Rev B 250413 BOM 250501.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimbuckett/Documents/Work/Smart Charger Files/Docs/BOMs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joris\Documents\GitHub\Externals-SmartCharger-Hardware\Smart Charger Files\Docs\BOMs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2070584D-7F0F-0242-9292-47A7810447ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE79267F-7E4F-4885-806E-93B45EDB6E66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9260" yWindow="500" windowWidth="40720" windowHeight="20820" xr2:uid="{FAF7EA74-0BDE-F041-9259-5544143833B1}"/>
+    <workbookView xWindow="10305" yWindow="2355" windowWidth="28020" windowHeight="16080" xr2:uid="{FAF7EA74-0BDE-F041-9259-5544143833B1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="754" uniqueCount="487">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="491">
   <si>
     <t>Item</t>
   </si>
@@ -395,9 +395,6 @@
     <t>445-6893-1-ND</t>
   </si>
   <si>
-    <t>C60, C61</t>
-  </si>
-  <si>
     <t>0.001uF</t>
   </si>
   <si>
@@ -1497,13 +1494,28 @@
   </si>
   <si>
     <t>Note</t>
+  </si>
+  <si>
+    <t>C61</t>
+  </si>
+  <si>
+    <t>C60</t>
+  </si>
+  <si>
+    <t>CAP CER 0.1uF 50V X7R 0603</t>
+  </si>
+  <si>
+    <t>GCM188R71H104KA57J</t>
+  </si>
+  <si>
+    <t>490-8020-1-ND</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1551,15 +1563,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF9C0006"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1569,11 +1574,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -1586,13 +1586,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1620,18 +1619,11 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
-  <cellStyles count="4">
-    <cellStyle name="Bad" xfId="3" builtinId="27"/>
+  <cellStyles count="3">
     <cellStyle name="Good" xfId="1" builtinId="26"/>
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1966,25 +1958,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36D0D730-67A9-204E-8F26-0B51C94EDA82}">
-  <dimension ref="A1:M101"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:M102"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.83203125" style="11" customWidth="1"/>
-    <col min="2" max="2" width="4.83203125" customWidth="1"/>
-    <col min="3" max="3" width="1.83203125" customWidth="1"/>
+    <col min="1" max="1" width="4.875" style="11" customWidth="1"/>
+    <col min="2" max="2" width="4.875" customWidth="1"/>
+    <col min="3" max="3" width="1.875" customWidth="1"/>
     <col min="4" max="4" width="37.5" customWidth="1"/>
-    <col min="5" max="5" width="21.1640625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="21.125" style="2" customWidth="1"/>
     <col min="6" max="6" width="52.5" customWidth="1"/>
-    <col min="7" max="7" width="13.83203125" customWidth="1"/>
-    <col min="8" max="8" width="21.83203125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="13.875" customWidth="1"/>
+    <col min="8" max="8" width="21.875" style="2" customWidth="1"/>
     <col min="9" max="9" width="7" customWidth="1"/>
-    <col min="10" max="10" width="27.83203125" customWidth="1"/>
+    <col min="10" max="10" width="27.875" customWidth="1"/>
     <col min="11" max="11" width="56.5" customWidth="1"/>
     <col min="12" max="12" width="4.5" style="1" customWidth="1"/>
-    <col min="13" max="13" width="23.33203125" customWidth="1"/>
+    <col min="13" max="13" width="23.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -2019,10 +2011,10 @@
         <v>10</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>486</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="11">
         <v>1</v>
       </c>
@@ -2057,7 +2049,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -2077,13 +2069,13 @@
         <v>23</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="I4" t="s">
         <v>16</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="K4" t="s">
         <v>24</v>
@@ -2092,7 +2084,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="11">
         <v>3</v>
       </c>
@@ -2124,7 +2116,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="11">
         <v>4</v>
       </c>
@@ -2156,7 +2148,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="11">
         <v>5</v>
       </c>
@@ -2188,7 +2180,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="11">
         <v>6</v>
       </c>
@@ -2220,7 +2212,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
         <v>7</v>
       </c>
@@ -2252,7 +2244,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="12">
         <v>8</v>
       </c>
@@ -2284,7 +2276,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="12">
         <v>9</v>
       </c>
@@ -2316,7 +2308,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="11">
         <v>10</v>
       </c>
@@ -2351,7 +2343,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
         <v>11</v>
       </c>
@@ -2383,7 +2375,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="11">
         <v>12</v>
       </c>
@@ -2415,7 +2407,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="11">
         <v>13</v>
       </c>
@@ -2447,7 +2439,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="11">
         <v>14</v>
       </c>
@@ -2479,7 +2471,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="11">
         <v>15</v>
       </c>
@@ -2511,7 +2503,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
         <v>16</v>
       </c>
@@ -2543,7 +2535,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="11">
         <v>17</v>
       </c>
@@ -2575,7 +2567,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="11">
         <v>18</v>
       </c>
@@ -2607,7 +2599,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="11">
         <v>19</v>
       </c>
@@ -2639,39 +2631,39 @@
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="11">
         <v>20</v>
       </c>
       <c r="B22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D22" t="s">
+        <v>486</v>
+      </c>
+      <c r="E22" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="F22" t="s">
         <v>120</v>
-      </c>
-      <c r="F22" t="s">
-        <v>121</v>
       </c>
       <c r="G22" t="s">
         <v>28</v>
       </c>
       <c r="H22" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="I22" t="s">
+        <v>16</v>
+      </c>
+      <c r="J22" s="3" t="s">
         <v>122</v>
-      </c>
-      <c r="I22" t="s">
-        <v>16</v>
-      </c>
-      <c r="J22" s="3" t="s">
-        <v>123</v>
       </c>
       <c r="K22" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
         <v>21</v>
       </c>
@@ -2679,31 +2671,31 @@
         <v>1</v>
       </c>
       <c r="D23" t="s">
-        <v>124</v>
+        <v>487</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>125</v>
+        <v>26</v>
       </c>
       <c r="F23" t="s">
-        <v>126</v>
+        <v>488</v>
       </c>
       <c r="G23" t="s">
-        <v>127</v>
+        <v>28</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>128</v>
+        <v>489</v>
       </c>
       <c r="I23" t="s">
         <v>16</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>129</v>
+        <v>490</v>
       </c>
       <c r="K23" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="11">
         <v>22</v>
       </c>
@@ -2711,31 +2703,31 @@
         <v>1</v>
       </c>
       <c r="D24" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="F24" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="G24" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="I24" t="s">
         <v>16</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="K24" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
         <v>23</v>
       </c>
@@ -2743,92 +2735,89 @@
         <v>1</v>
       </c>
       <c r="D25" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="F25" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="G25" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="I25" t="s">
         <v>16</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="K25" t="s">
-        <v>142</v>
-      </c>
-      <c r="L25" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="11">
         <v>24</v>
       </c>
       <c r="B26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D26" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="F26" t="s">
-        <v>145</v>
+        <v>137</v>
+      </c>
+      <c r="G26" t="s">
+        <v>138</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="I26" t="s">
+        <v>16</v>
+      </c>
+      <c r="J26" s="3" t="s">
+        <v>140</v>
       </c>
       <c r="K26" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="L26" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
         <v>25</v>
       </c>
       <c r="B27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D27" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="F27" t="s">
-        <v>149</v>
-      </c>
-      <c r="G27" t="s">
-        <v>139</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="I27" t="s">
-        <v>16</v>
-      </c>
-      <c r="J27" s="3" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="K27" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="L27" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="11">
         <v>26</v>
       </c>
@@ -2836,89 +2825,92 @@
         <v>1</v>
       </c>
       <c r="D28" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="F28" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="G28" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="I28" t="s">
         <v>16</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="K28" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="L28" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
         <v>27</v>
       </c>
       <c r="B29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="F29" t="s">
-        <v>157</v>
+        <v>152</v>
+      </c>
+      <c r="G29" t="s">
+        <v>138</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="I29" t="s">
+        <v>16</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>154</v>
       </c>
       <c r="K29" t="s">
-        <v>158</v>
+        <v>141</v>
       </c>
       <c r="L29" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A30" s="1">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A30" s="11">
         <v>28</v>
       </c>
       <c r="B30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D30" t="s">
-        <v>459</v>
+        <v>155</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>460</v>
+        <v>136</v>
       </c>
       <c r="F30" t="s">
-        <v>461</v>
-      </c>
-      <c r="G30" t="s">
-        <v>309</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>460</v>
-      </c>
-      <c r="I30" t="s">
-        <v>16</v>
-      </c>
-      <c r="J30" s="3" t="s">
-        <v>462</v>
+        <v>156</v>
       </c>
       <c r="K30" t="s">
-        <v>485</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+        <v>157</v>
+      </c>
+      <c r="L30" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
         <v>29</v>
       </c>
@@ -2926,22 +2918,31 @@
         <v>1</v>
       </c>
       <c r="D31" t="s">
-        <v>159</v>
+        <v>458</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>160</v>
+        <v>459</v>
       </c>
       <c r="F31" t="s">
-        <v>161</v>
+        <v>460</v>
+      </c>
+      <c r="G31" t="s">
+        <v>308</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="I31" t="s">
+        <v>16</v>
+      </c>
+      <c r="J31" s="3" t="s">
+        <v>461</v>
       </c>
       <c r="K31" t="s">
-        <v>162</v>
-      </c>
-      <c r="L31" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="11">
         <v>30</v>
       </c>
@@ -2949,221 +2950,212 @@
         <v>1</v>
       </c>
       <c r="D32" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="F32" t="s">
-        <v>165</v>
-      </c>
-      <c r="G32" t="s">
-        <v>166</v>
-      </c>
-      <c r="H32" s="14">
-        <v>3568</v>
-      </c>
-      <c r="I32" t="s">
-        <v>16</v>
-      </c>
-      <c r="J32" s="3" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="K32" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="L32" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="11">
         <v>31</v>
       </c>
       <c r="B33">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D33" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="H33" s="7"/>
-      <c r="J33" s="3"/>
+        <v>163</v>
+      </c>
+      <c r="F33" t="s">
+        <v>164</v>
+      </c>
+      <c r="G33" t="s">
+        <v>165</v>
+      </c>
+      <c r="H33" s="7">
+        <v>3568</v>
+      </c>
+      <c r="I33" t="s">
+        <v>16</v>
+      </c>
+      <c r="J33" s="3" t="s">
+        <v>166</v>
+      </c>
       <c r="K33" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="L33" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="11">
         <v>32</v>
       </c>
       <c r="B34">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D34" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>173</v>
-      </c>
+        <v>169</v>
+      </c>
+      <c r="H34" s="7"/>
+      <c r="J34" s="3"/>
       <c r="K34" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="L34" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="11">
         <v>33</v>
       </c>
       <c r="B35">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D35" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="E35" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="K35" t="s">
         <v>173</v>
-      </c>
-      <c r="K35" t="s">
-        <v>176</v>
       </c>
       <c r="L35" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
         <v>34</v>
       </c>
       <c r="B36">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D36" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="F36" t="s">
-        <v>179</v>
-      </c>
-      <c r="G36" t="s">
-        <v>180</v>
-      </c>
-      <c r="H36" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="I36" t="s">
-        <v>16</v>
-      </c>
-      <c r="J36" s="3" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="K36" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="L36" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="11">
         <v>35</v>
       </c>
       <c r="B37">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D37" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="F37" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="G37" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="I37" t="s">
         <v>16</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="K37" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="L37" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A38" s="12">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A38" s="11">
         <v>36</v>
       </c>
       <c r="B38">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="D38" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="F38" t="s">
-        <v>193</v>
+        <v>185</v>
+      </c>
+      <c r="G38" t="s">
+        <v>186</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="I38" t="s">
+        <v>16</v>
+      </c>
+      <c r="J38" s="3" t="s">
+        <v>188</v>
       </c>
       <c r="K38" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="L38" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="11">
         <v>37</v>
       </c>
       <c r="B39">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D39" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="F39" t="s">
-        <v>197</v>
-      </c>
-      <c r="G39" t="s">
-        <v>198</v>
-      </c>
-      <c r="H39" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="I39" t="s">
-        <v>16</v>
-      </c>
-      <c r="J39" s="3" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="K39" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
+        <v>193</v>
+      </c>
+      <c r="L39" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="11">
         <v>38</v>
       </c>
@@ -3171,34 +3163,31 @@
         <v>1</v>
       </c>
       <c r="D40" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="F40" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="G40" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="I40" t="s">
         <v>16</v>
       </c>
       <c r="J40" s="3" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="K40" t="s">
-        <v>206</v>
-      </c>
-      <c r="L40" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
         <v>39</v>
       </c>
@@ -3206,34 +3195,34 @@
         <v>1</v>
       </c>
       <c r="D41" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="F41" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="G41" t="s">
-        <v>210</v>
-      </c>
-      <c r="H41" s="14">
-        <v>901303112</v>
+        <v>203</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>201</v>
       </c>
       <c r="I41" t="s">
         <v>16</v>
       </c>
       <c r="J41" s="3" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="K41" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="L41" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" s="11">
         <v>40</v>
       </c>
@@ -3241,34 +3230,34 @@
         <v>1</v>
       </c>
       <c r="D42" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="F42" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="G42" t="s">
-        <v>216</v>
-      </c>
-      <c r="H42" s="2" t="s">
-        <v>217</v>
+        <v>209</v>
+      </c>
+      <c r="H42" s="7">
+        <v>901303112</v>
       </c>
       <c r="I42" t="s">
-        <v>218</v>
+        <v>16</v>
       </c>
       <c r="J42" s="3" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="K42" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="L42" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
         <v>41</v>
       </c>
@@ -3276,139 +3265,139 @@
         <v>1</v>
       </c>
       <c r="D43" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="F43" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
       <c r="G43" t="s">
-        <v>210</v>
-      </c>
-      <c r="H43" s="14">
-        <v>901301306</v>
+        <v>215</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>216</v>
       </c>
       <c r="I43" t="s">
-        <v>16</v>
+        <v>217</v>
       </c>
       <c r="J43" s="3" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="K43" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="L43" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" s="11">
         <v>42</v>
       </c>
       <c r="B44">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D44" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="F44" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="G44" t="s">
-        <v>187</v>
-      </c>
-      <c r="H44" s="2" t="s">
-        <v>229</v>
+        <v>209</v>
+      </c>
+      <c r="H44" s="7">
+        <v>901301306</v>
       </c>
       <c r="I44" t="s">
         <v>16</v>
       </c>
       <c r="J44" s="3" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="K44" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="L44" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
         <v>43</v>
       </c>
       <c r="B45">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D45" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="E45" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="F45" t="s">
         <v>227</v>
       </c>
-      <c r="F45" t="s">
-        <v>233</v>
-      </c>
       <c r="G45" t="s">
-        <v>216</v>
+        <v>186</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="I45" t="s">
         <v>16</v>
       </c>
       <c r="J45" s="3" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="K45" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="L45" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" s="11">
         <v>44</v>
       </c>
       <c r="B46">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D46" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>238</v>
+        <v>226</v>
       </c>
       <c r="F46" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="G46" t="s">
-        <v>210</v>
-      </c>
-      <c r="H46" s="14">
-        <v>901361106</v>
+        <v>215</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>233</v>
       </c>
       <c r="I46" t="s">
         <v>16</v>
       </c>
       <c r="J46" s="3" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="K46" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="L46" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" s="11">
         <v>45</v>
       </c>
@@ -3416,34 +3405,34 @@
         <v>1</v>
       </c>
       <c r="D47" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="F47" t="s">
-        <v>243</v>
+        <v>222</v>
       </c>
       <c r="G47" t="s">
-        <v>187</v>
-      </c>
-      <c r="H47" s="2" t="s">
-        <v>244</v>
+        <v>209</v>
+      </c>
+      <c r="H47" s="7">
+        <v>901361106</v>
       </c>
       <c r="I47" t="s">
         <v>16</v>
       </c>
       <c r="J47" s="3" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="K47" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="L47" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
         <v>46</v>
       </c>
@@ -3451,34 +3440,34 @@
         <v>1</v>
       </c>
       <c r="D48" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="F48" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="G48" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="I48" t="s">
         <v>16</v>
       </c>
       <c r="J48" s="3" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="K48" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="L48" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" s="11">
         <v>47</v>
       </c>
@@ -3486,34 +3475,34 @@
         <v>1</v>
       </c>
       <c r="D49" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="F49" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="G49" t="s">
-        <v>210</v>
-      </c>
-      <c r="H49" s="7">
-        <v>901303108</v>
+        <v>186</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>249</v>
       </c>
       <c r="I49" t="s">
         <v>16</v>
       </c>
       <c r="J49" s="3" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="K49" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="L49" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
         <v>48</v>
       </c>
@@ -3521,34 +3510,34 @@
         <v>1</v>
       </c>
       <c r="D50" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>227</v>
+        <v>253</v>
       </c>
       <c r="F50" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="G50" t="s">
-        <v>216</v>
-      </c>
-      <c r="H50" s="2" t="s">
-        <v>260</v>
+        <v>209</v>
+      </c>
+      <c r="H50" s="7">
+        <v>901303108</v>
       </c>
       <c r="I50" t="s">
         <v>16</v>
       </c>
       <c r="J50" s="3" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="K50" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="L50" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" s="11">
         <v>49</v>
       </c>
@@ -3556,34 +3545,34 @@
         <v>1</v>
       </c>
       <c r="D51" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>264</v>
+        <v>226</v>
       </c>
       <c r="F51" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="G51" t="s">
-        <v>210</v>
-      </c>
-      <c r="H51" s="14">
-        <v>901361104</v>
+        <v>215</v>
+      </c>
+      <c r="H51" s="2" t="s">
+        <v>259</v>
       </c>
       <c r="I51" t="s">
         <v>16</v>
       </c>
       <c r="J51" s="3" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="K51" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="L51" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
         <v>50</v>
       </c>
@@ -3591,203 +3580,206 @@
         <v>1</v>
       </c>
       <c r="D52" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>227</v>
+        <v>263</v>
       </c>
       <c r="F52" t="s">
-        <v>228</v>
+        <v>264</v>
       </c>
       <c r="G52" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H52" s="7">
-        <v>901361102</v>
+        <v>901361104</v>
       </c>
       <c r="I52" t="s">
         <v>16</v>
       </c>
       <c r="J52" s="3" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="K52" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="L52" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A53" s="11">
         <v>51</v>
       </c>
       <c r="B53">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D53" t="s">
-        <v>271</v>
-      </c>
-      <c r="E53" s="2">
-        <v>0.156</v>
+        <v>267</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>226</v>
       </c>
       <c r="F53" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="G53" t="s">
-        <v>216</v>
-      </c>
-      <c r="H53" s="2" t="s">
-        <v>272</v>
+        <v>209</v>
+      </c>
+      <c r="H53" s="7">
+        <v>901361102</v>
       </c>
       <c r="I53" t="s">
         <v>16</v>
       </c>
       <c r="J53" s="3" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="K53" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="L53" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54" s="11">
         <v>52</v>
       </c>
       <c r="B54">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D54" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="E54" s="2">
-        <v>0.1</v>
+        <v>0.156</v>
       </c>
       <c r="F54" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="G54" t="s">
-        <v>187</v>
+        <v>215</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>229</v>
+        <v>271</v>
       </c>
       <c r="I54" t="s">
         <v>16</v>
       </c>
       <c r="J54" s="3" t="s">
-        <v>230</v>
+        <v>272</v>
       </c>
       <c r="K54" t="s">
-        <v>231</v>
+        <v>273</v>
       </c>
       <c r="L54" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
         <v>53</v>
       </c>
       <c r="B55">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D55" t="s">
-        <v>276</v>
-      </c>
-      <c r="E55" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="E55" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="F55" t="s">
         <v>227</v>
       </c>
-      <c r="F55" t="s">
-        <v>277</v>
-      </c>
       <c r="G55" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>278</v>
+        <v>228</v>
       </c>
       <c r="I55" t="s">
         <v>16</v>
       </c>
       <c r="J55" s="3" t="s">
-        <v>279</v>
+        <v>229</v>
       </c>
       <c r="K55" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="L55" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A56" s="11">
         <v>54</v>
       </c>
       <c r="B56">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D56" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>281</v>
-      </c>
-      <c r="F56" s="4" t="s">
-        <v>282</v>
-      </c>
-      <c r="G56" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="H56" s="7" t="s">
-        <v>284</v>
-      </c>
-      <c r="I56" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="J56" s="5" t="s">
-        <v>285</v>
+        <v>226</v>
+      </c>
+      <c r="F56" t="s">
+        <v>276</v>
+      </c>
+      <c r="G56" t="s">
+        <v>186</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="I56" t="s">
+        <v>16</v>
+      </c>
+      <c r="J56" s="3" t="s">
+        <v>278</v>
       </c>
       <c r="K56" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
+        <v>230</v>
+      </c>
+      <c r="L56" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
         <v>55</v>
       </c>
       <c r="B57">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D57" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="F57" t="s">
-        <v>289</v>
+        <v>280</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>281</v>
       </c>
       <c r="G57" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="H57" s="7" t="s">
         <v>283</v>
       </c>
-      <c r="H57" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="I57" t="s">
-        <v>16</v>
-      </c>
-      <c r="J57" s="3" t="s">
-        <v>291</v>
+      <c r="I57" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="J57" s="5" t="s">
+        <v>284</v>
       </c>
       <c r="K57" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A58" s="11">
         <v>56</v>
       </c>
@@ -3795,191 +3787,191 @@
         <v>2</v>
       </c>
       <c r="D58" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="F58" t="s">
-        <v>295</v>
-      </c>
-      <c r="G58" t="s">
-        <v>296</v>
+        <v>288</v>
+      </c>
+      <c r="G58" s="4" t="s">
+        <v>282</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="I58" t="s">
         <v>16</v>
       </c>
       <c r="J58" s="3" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="K58" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
         <v>57</v>
       </c>
       <c r="B59">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D59" t="s">
-        <v>300</v>
+        <v>292</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>301</v>
+        <v>293</v>
       </c>
       <c r="F59" t="s">
-        <v>302</v>
+        <v>294</v>
       </c>
       <c r="G59" t="s">
-        <v>303</v>
+        <v>295</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="I59" t="s">
         <v>16</v>
       </c>
       <c r="J59" s="3" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="K59" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A60" s="11">
         <v>58</v>
       </c>
       <c r="B60">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D60" t="s">
-        <v>306</v>
+        <v>299</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="F60" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
       <c r="G60" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="I60" t="s">
         <v>16</v>
       </c>
       <c r="J60" s="3" t="s">
-        <v>311</v>
+        <v>303</v>
       </c>
       <c r="K60" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
         <v>59</v>
       </c>
       <c r="B61">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D61" t="s">
-        <v>312</v>
+        <v>305</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="F61" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="G61" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
       <c r="H61" s="2" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
       <c r="I61" t="s">
         <v>16</v>
       </c>
       <c r="J61" s="3" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="K61" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A62" s="11">
         <v>60</v>
       </c>
       <c r="B62">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D62" t="s">
-        <v>319</v>
-      </c>
-      <c r="E62" s="2">
-        <v>10</v>
+        <v>311</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>312</v>
       </c>
       <c r="F62" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="G62" t="s">
+        <v>314</v>
+      </c>
+      <c r="H62" s="2" t="s">
         <v>315</v>
       </c>
-      <c r="H62" s="2" t="s">
-        <v>321</v>
-      </c>
       <c r="I62" t="s">
         <v>16</v>
       </c>
       <c r="J62" s="3" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="K62" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
         <v>61</v>
       </c>
       <c r="B63">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D63" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="E63" s="2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F63" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="G63" t="s">
-        <v>61</v>
+        <v>314</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="I63" t="s">
         <v>16</v>
       </c>
       <c r="J63" s="3" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="K63" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A64" s="11">
         <v>62</v>
       </c>
@@ -3987,31 +3979,31 @@
         <v>1</v>
       </c>
       <c r="D64" t="s">
-        <v>328</v>
-      </c>
-      <c r="E64" s="2" t="s">
-        <v>329</v>
+        <v>322</v>
+      </c>
+      <c r="E64" s="2">
+        <v>0</v>
       </c>
       <c r="F64" t="s">
-        <v>330</v>
+        <v>323</v>
       </c>
       <c r="G64" t="s">
-        <v>315</v>
+        <v>61</v>
       </c>
       <c r="H64" s="2" t="s">
-        <v>331</v>
+        <v>324</v>
       </c>
       <c r="I64" t="s">
         <v>16</v>
       </c>
       <c r="J64" s="3" t="s">
-        <v>332</v>
+        <v>325</v>
       </c>
       <c r="K64" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.2">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
         <v>63</v>
       </c>
@@ -4019,351 +4011,351 @@
         <v>1</v>
       </c>
       <c r="D65" t="s">
-        <v>333</v>
-      </c>
-      <c r="E65" t="s">
-        <v>334</v>
+        <v>327</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>328</v>
       </c>
       <c r="F65" t="s">
-        <v>335</v>
+        <v>329</v>
       </c>
       <c r="G65" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H65" s="2" t="s">
-        <v>336</v>
+        <v>330</v>
       </c>
       <c r="I65" t="s">
         <v>16</v>
       </c>
       <c r="J65" s="3" t="s">
-        <v>337</v>
+        <v>331</v>
       </c>
       <c r="K65" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.2">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="11">
         <v>64</v>
       </c>
       <c r="B66">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D66" t="s">
-        <v>338</v>
-      </c>
-      <c r="E66" s="2" t="s">
-        <v>339</v>
+        <v>332</v>
+      </c>
+      <c r="E66" t="s">
+        <v>333</v>
       </c>
       <c r="F66" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="G66" t="s">
-        <v>341</v>
+        <v>314</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="I66" t="s">
         <v>16</v>
       </c>
-      <c r="J66" s="6" t="s">
-        <v>342</v>
+      <c r="J66" s="3" t="s">
+        <v>336</v>
       </c>
       <c r="K66" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.2">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
         <v>65</v>
       </c>
       <c r="B67">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D67" t="s">
-        <v>344</v>
+        <v>337</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>345</v>
+        <v>338</v>
       </c>
       <c r="F67" t="s">
-        <v>346</v>
+        <v>339</v>
       </c>
       <c r="G67" t="s">
-        <v>315</v>
+        <v>340</v>
       </c>
       <c r="H67" s="2" t="s">
-        <v>347</v>
+        <v>338</v>
       </c>
       <c r="I67" t="s">
         <v>16</v>
       </c>
-      <c r="J67" s="3" t="s">
-        <v>348</v>
+      <c r="J67" s="6" t="s">
+        <v>341</v>
       </c>
       <c r="K67" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.2">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="11">
         <v>66</v>
       </c>
       <c r="B68">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D68" t="s">
-        <v>349</v>
-      </c>
-      <c r="E68" s="2">
-        <v>10</v>
+        <v>343</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>344</v>
       </c>
       <c r="F68" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="G68" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H68" s="2" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="I68" t="s">
         <v>16</v>
       </c>
       <c r="J68" s="3" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="K68" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A69" s="13">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A69" s="11">
         <v>67</v>
       </c>
       <c r="B69">
         <v>2</v>
       </c>
       <c r="D69" t="s">
-        <v>353</v>
-      </c>
-      <c r="E69" s="2" t="s">
-        <v>354</v>
+        <v>348</v>
+      </c>
+      <c r="E69" s="2">
+        <v>10</v>
       </c>
       <c r="F69" t="s">
-        <v>355</v>
+        <v>349</v>
       </c>
       <c r="G69" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H69" s="2" t="s">
-        <v>356</v>
+        <v>350</v>
       </c>
       <c r="I69" t="s">
         <v>16</v>
       </c>
       <c r="J69" s="3" t="s">
-        <v>357</v>
+        <v>351</v>
       </c>
       <c r="K69" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.2">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="11">
         <v>68</v>
       </c>
       <c r="B70">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D70" t="s">
-        <v>358</v>
-      </c>
-      <c r="E70" s="2">
-        <v>100</v>
+        <v>352</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>353</v>
       </c>
       <c r="F70" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="G70" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H70" s="2" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="I70" t="s">
         <v>16</v>
       </c>
       <c r="J70" s="3" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="K70" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.2">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="11">
         <v>69</v>
       </c>
       <c r="B71">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D71" t="s">
-        <v>362</v>
-      </c>
-      <c r="E71" s="2" t="s">
-        <v>363</v>
+        <v>357</v>
+      </c>
+      <c r="E71" s="2">
+        <v>100</v>
       </c>
       <c r="F71" t="s">
-        <v>364</v>
+        <v>358</v>
       </c>
       <c r="G71" t="s">
-        <v>315</v>
-      </c>
-      <c r="H71" s="15" t="s">
-        <v>365</v>
+        <v>314</v>
+      </c>
+      <c r="H71" s="2" t="s">
+        <v>359</v>
       </c>
       <c r="I71" t="s">
         <v>16</v>
       </c>
       <c r="J71" s="3" t="s">
-        <v>366</v>
+        <v>360</v>
       </c>
       <c r="K71" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.2">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="11">
         <v>70</v>
       </c>
       <c r="B72">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D72" t="s">
-        <v>367</v>
+        <v>361</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>368</v>
+        <v>362</v>
       </c>
       <c r="F72" t="s">
-        <v>369</v>
+        <v>363</v>
       </c>
       <c r="G72" t="s">
-        <v>370</v>
-      </c>
-      <c r="H72" s="2" t="s">
-        <v>368</v>
+        <v>314</v>
+      </c>
+      <c r="H72" s="13" t="s">
+        <v>364</v>
       </c>
       <c r="I72" t="s">
         <v>16</v>
       </c>
       <c r="J72" s="3" t="s">
-        <v>371</v>
+        <v>365</v>
       </c>
       <c r="K72" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.2">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="11">
         <v>71</v>
       </c>
       <c r="B73">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D73" t="s">
-        <v>373</v>
+        <v>366</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>374</v>
+        <v>367</v>
       </c>
       <c r="F73" t="s">
-        <v>375</v>
+        <v>368</v>
       </c>
       <c r="G73" t="s">
+        <v>369</v>
+      </c>
+      <c r="H73" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="I73" t="s">
+        <v>16</v>
+      </c>
+      <c r="J73" s="3" t="s">
         <v>370</v>
       </c>
-      <c r="H73" s="2" t="s">
-        <v>374</v>
-      </c>
-      <c r="I73" t="s">
-        <v>16</v>
-      </c>
-      <c r="J73" s="6" t="s">
-        <v>376</v>
-      </c>
       <c r="K73" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.2">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="11">
         <v>72</v>
       </c>
       <c r="B74">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D74" t="s">
-        <v>378</v>
+        <v>372</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>379</v>
+        <v>373</v>
       </c>
       <c r="F74" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="G74" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
       <c r="H74" s="2" t="s">
-        <v>382</v>
+        <v>373</v>
       </c>
       <c r="I74" t="s">
         <v>16</v>
       </c>
-      <c r="J74" s="3" t="s">
-        <v>383</v>
+      <c r="J74" s="6" t="s">
+        <v>375</v>
       </c>
       <c r="K74" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.2">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="11">
         <v>73</v>
       </c>
       <c r="B75">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D75" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>386</v>
+        <v>378</v>
       </c>
       <c r="F75" t="s">
-        <v>387</v>
+        <v>379</v>
       </c>
       <c r="G75" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="H75" s="2" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="I75" t="s">
         <v>16</v>
       </c>
-      <c r="J75" s="6" t="s">
-        <v>390</v>
+      <c r="J75" s="3" t="s">
+        <v>382</v>
       </c>
       <c r="K75" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.2">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="11">
         <v>74</v>
       </c>
@@ -4371,63 +4363,63 @@
         <v>1</v>
       </c>
       <c r="D76" t="s">
+        <v>384</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="F76" t="s">
+        <v>386</v>
+      </c>
+      <c r="G76" t="s">
+        <v>387</v>
+      </c>
+      <c r="H76" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="I76" t="s">
+        <v>16</v>
+      </c>
+      <c r="J76" s="6" t="s">
+        <v>389</v>
+      </c>
+      <c r="K76" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A77" s="11">
+        <v>75</v>
+      </c>
+      <c r="B77">
+        <v>1</v>
+      </c>
+      <c r="D77" t="s">
+        <v>391</v>
+      </c>
+      <c r="E77" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="E76" s="2" t="s">
+      <c r="F77" t="s">
         <v>393</v>
       </c>
-      <c r="F76" t="s">
+      <c r="G77" t="s">
+        <v>369</v>
+      </c>
+      <c r="H77" s="2" t="s">
         <v>394</v>
       </c>
-      <c r="G76" t="s">
-        <v>370</v>
-      </c>
-      <c r="H76" s="2" t="s">
+      <c r="I77" t="s">
+        <v>16</v>
+      </c>
+      <c r="J77" s="3" t="s">
         <v>395</v>
       </c>
-      <c r="I76" t="s">
-        <v>16</v>
-      </c>
-      <c r="J76" s="3" t="s">
+      <c r="K77" t="s">
         <v>396</v>
       </c>
-      <c r="K76" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A77" s="12">
-        <v>75</v>
-      </c>
-      <c r="B77">
-        <v>1</v>
-      </c>
-      <c r="D77" t="s">
-        <v>398</v>
-      </c>
-      <c r="E77" s="2" t="s">
-        <v>399</v>
-      </c>
-      <c r="F77" t="s">
-        <v>400</v>
-      </c>
-      <c r="G77" t="s">
-        <v>381</v>
-      </c>
-      <c r="H77" s="2" t="s">
-        <v>399</v>
-      </c>
-      <c r="I77" t="s">
-        <v>16</v>
-      </c>
-      <c r="J77" s="3" t="s">
-        <v>401</v>
-      </c>
-      <c r="K77" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="11">
         <v>76</v>
       </c>
@@ -4435,31 +4427,31 @@
         <v>1</v>
       </c>
       <c r="D78" t="s">
-        <v>403</v>
+        <v>397</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>404</v>
+        <v>398</v>
       </c>
       <c r="F78" t="s">
-        <v>405</v>
+        <v>399</v>
       </c>
       <c r="G78" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H78" s="2" t="s">
-        <v>406</v>
+        <v>398</v>
       </c>
       <c r="I78" t="s">
         <v>16</v>
       </c>
       <c r="J78" s="3" t="s">
-        <v>407</v>
+        <v>400</v>
       </c>
       <c r="K78" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.2">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="11">
         <v>77</v>
       </c>
@@ -4467,31 +4459,31 @@
         <v>1</v>
       </c>
       <c r="D79" t="s">
-        <v>409</v>
+        <v>402</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>410</v>
+        <v>403</v>
       </c>
       <c r="F79" t="s">
-        <v>411</v>
+        <v>404</v>
       </c>
       <c r="G79" t="s">
-        <v>370</v>
+        <v>380</v>
       </c>
       <c r="H79" s="2" t="s">
-        <v>412</v>
+        <v>405</v>
       </c>
       <c r="I79" t="s">
         <v>16</v>
       </c>
       <c r="J79" s="3" t="s">
-        <v>413</v>
+        <v>406</v>
       </c>
       <c r="K79" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.2">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="11">
         <v>78</v>
       </c>
@@ -4499,34 +4491,31 @@
         <v>1</v>
       </c>
       <c r="D80" t="s">
-        <v>463</v>
+        <v>408</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>164</v>
+        <v>409</v>
       </c>
       <c r="F80" t="s">
-        <v>415</v>
+        <v>410</v>
       </c>
       <c r="G80" t="s">
-        <v>416</v>
+        <v>369</v>
       </c>
       <c r="H80" s="2" t="s">
-        <v>417</v>
+        <v>411</v>
       </c>
       <c r="I80" t="s">
         <v>16</v>
       </c>
       <c r="J80" s="3" t="s">
-        <v>418</v>
+        <v>412</v>
       </c>
       <c r="K80" t="s">
-        <v>162</v>
-      </c>
-      <c r="L80" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.2">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="81" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A81" s="11">
         <v>79</v>
       </c>
@@ -4534,37 +4523,34 @@
         <v>1</v>
       </c>
       <c r="D81" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>419</v>
+        <v>163</v>
       </c>
       <c r="F81" t="s">
-        <v>420</v>
+        <v>414</v>
       </c>
       <c r="G81" t="s">
-        <v>421</v>
+        <v>415</v>
       </c>
       <c r="H81" s="2" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="I81" t="s">
         <v>16</v>
       </c>
       <c r="J81" s="3" t="s">
-        <v>423</v>
+        <v>417</v>
       </c>
       <c r="K81" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L81" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="M81" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.2">
+    </row>
+    <row r="82" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A82" s="11">
         <v>80</v>
       </c>
@@ -4572,34 +4558,37 @@
         <v>1</v>
       </c>
       <c r="D82" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="E82" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="F82" t="s">
         <v>419</v>
       </c>
-      <c r="F82" t="s">
-        <v>424</v>
-      </c>
       <c r="G82" t="s">
-        <v>210</v>
-      </c>
-      <c r="H82" s="2">
-        <v>901420012</v>
+        <v>420</v>
+      </c>
+      <c r="H82" s="2" t="s">
+        <v>421</v>
       </c>
       <c r="I82" t="s">
         <v>16</v>
       </c>
       <c r="J82" s="3" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="K82" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L82" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="M82" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="83" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A83" s="11">
         <v>81</v>
       </c>
@@ -4607,37 +4596,34 @@
         <v>1</v>
       </c>
       <c r="D83" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="F83" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="G83" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H83" s="2">
-        <v>901420006</v>
+        <v>901420012</v>
       </c>
       <c r="I83" t="s">
         <v>16</v>
       </c>
       <c r="J83" s="3" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="K83" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L83" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="M83" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="84" spans="1:13" x14ac:dyDescent="0.2">
+    </row>
+    <row r="84" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A84" s="11">
         <v>82</v>
       </c>
@@ -4645,37 +4631,37 @@
         <v>1</v>
       </c>
       <c r="D84" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="F84" t="s">
+        <v>425</v>
+      </c>
+      <c r="G84" t="s">
+        <v>209</v>
+      </c>
+      <c r="H84" s="2">
+        <v>901420006</v>
+      </c>
+      <c r="I84" t="s">
+        <v>16</v>
+      </c>
+      <c r="J84" s="3" t="s">
         <v>426</v>
       </c>
-      <c r="G84" t="s">
-        <v>210</v>
-      </c>
-      <c r="H84" s="2">
-        <v>901560146</v>
-      </c>
-      <c r="I84" t="s">
-        <v>16</v>
-      </c>
-      <c r="J84" s="3" t="s">
-        <v>428</v>
-      </c>
       <c r="K84" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L84" s="1" t="s">
         <v>19</v>
       </c>
       <c r="M84" t="s">
-        <v>479</v>
-      </c>
-    </row>
-    <row r="85" spans="1:13" x14ac:dyDescent="0.2">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="85" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A85" s="11">
         <v>83</v>
       </c>
@@ -4683,113 +4669,113 @@
         <v>1</v>
       </c>
       <c r="D85" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="F85" t="s">
-        <v>429</v>
+        <v>425</v>
       </c>
       <c r="G85" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H85" s="2">
-        <v>901420008</v>
+        <v>901560146</v>
       </c>
       <c r="I85" t="s">
         <v>16</v>
       </c>
       <c r="J85" s="3" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="K85" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L85" s="1" t="s">
         <v>19</v>
       </c>
       <c r="M85" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="86" spans="1:13" x14ac:dyDescent="0.2">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="86" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A86" s="11">
         <v>84</v>
       </c>
       <c r="B86">
-        <v>2</v>
-      </c>
-      <c r="D86" s="8" t="s">
-        <v>469</v>
-      </c>
-      <c r="E86" s="9" t="s">
-        <v>419</v>
+        <v>1</v>
+      </c>
+      <c r="D86" t="s">
+        <v>467</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>418</v>
       </c>
       <c r="F86" t="s">
-        <v>431</v>
-      </c>
-      <c r="G86" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="H86" s="8" t="s">
-        <v>432</v>
-      </c>
-      <c r="I86" s="9" t="s">
+        <v>428</v>
+      </c>
+      <c r="G86" t="s">
+        <v>209</v>
+      </c>
+      <c r="H86" s="2">
+        <v>901420008</v>
+      </c>
+      <c r="I86" t="s">
         <v>16</v>
       </c>
       <c r="J86" s="3" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
       <c r="K86" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L86" s="1" t="s">
         <v>19</v>
       </c>
       <c r="M86" t="s">
-        <v>481</v>
-      </c>
-    </row>
-    <row r="87" spans="1:13" x14ac:dyDescent="0.2">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="87" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A87" s="11">
         <v>85</v>
       </c>
       <c r="B87">
-        <v>1</v>
-      </c>
-      <c r="D87" t="s">
-        <v>470</v>
-      </c>
-      <c r="E87" s="2" t="s">
-        <v>419</v>
+        <v>2</v>
+      </c>
+      <c r="D87" s="8" t="s">
+        <v>468</v>
+      </c>
+      <c r="E87" s="9" t="s">
+        <v>418</v>
       </c>
       <c r="F87" t="s">
-        <v>434</v>
-      </c>
-      <c r="G87" t="s">
-        <v>187</v>
-      </c>
-      <c r="H87" s="2" t="s">
-        <v>435</v>
-      </c>
-      <c r="I87" t="s">
+        <v>430</v>
+      </c>
+      <c r="G87" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="H87" s="8" t="s">
+        <v>431</v>
+      </c>
+      <c r="I87" s="9" t="s">
         <v>16</v>
       </c>
       <c r="J87" s="3" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="K87" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L87" s="1" t="s">
         <v>19</v>
       </c>
       <c r="M87" t="s">
-        <v>481</v>
-      </c>
-    </row>
-    <row r="88" spans="1:13" x14ac:dyDescent="0.2">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="88" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A88" s="11">
         <v>86</v>
       </c>
@@ -4797,275 +4783,313 @@
         <v>1</v>
       </c>
       <c r="D88" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="F88" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="G88" t="s">
-        <v>210</v>
-      </c>
-      <c r="H88" s="2">
-        <v>901560144</v>
+        <v>186</v>
+      </c>
+      <c r="H88" s="2" t="s">
+        <v>434</v>
       </c>
       <c r="I88" t="s">
         <v>16</v>
       </c>
       <c r="J88" s="3" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="K88" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L88" s="1" t="s">
         <v>19</v>
       </c>
       <c r="M88" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="89" spans="1:13" x14ac:dyDescent="0.2">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="89" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A89" s="11">
         <v>87</v>
       </c>
       <c r="B89">
         <v>1</v>
       </c>
-      <c r="D89" s="4" t="s">
-        <v>472</v>
+      <c r="D89" t="s">
+        <v>470</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="F89" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="G89" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H89" s="2">
-        <v>901560142</v>
+        <v>901560144</v>
       </c>
       <c r="I89" t="s">
         <v>16</v>
       </c>
       <c r="J89" s="3" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="K89" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L89" s="1" t="s">
         <v>19</v>
       </c>
       <c r="M89" t="s">
-        <v>483</v>
-      </c>
-    </row>
-    <row r="90" spans="1:13" x14ac:dyDescent="0.2">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="90" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A90" s="11">
         <v>88</v>
       </c>
       <c r="B90">
-        <v>30</v>
-      </c>
-      <c r="D90" t="s">
-        <v>484</v>
+        <v>1</v>
+      </c>
+      <c r="D90" s="4" t="s">
+        <v>471</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="F90" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="G90" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H90" s="2">
-        <v>901192110</v>
+        <v>901560142</v>
       </c>
       <c r="I90" t="s">
         <v>16</v>
       </c>
       <c r="J90" s="3" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
       <c r="K90" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L90" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="91" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="M90" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="91" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A91" s="11">
         <v>89</v>
       </c>
       <c r="B91">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="D91" t="s">
-        <v>476</v>
+        <v>483</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="F91" t="s">
-        <v>445</v>
+        <v>441</v>
       </c>
       <c r="G91" t="s">
-        <v>216</v>
-      </c>
-      <c r="H91" s="2" t="s">
-        <v>446</v>
+        <v>209</v>
+      </c>
+      <c r="H91" s="2">
+        <v>901192110</v>
       </c>
       <c r="I91" t="s">
         <v>16</v>
       </c>
       <c r="J91" s="3" t="s">
-        <v>447</v>
+        <v>442</v>
       </c>
       <c r="K91" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L91" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="92" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A92" s="11">
         <v>90</v>
       </c>
       <c r="B92">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D92" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="E92" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="F92" t="s">
         <v>444</v>
       </c>
-      <c r="F92" s="10" t="s">
-        <v>448</v>
-      </c>
       <c r="G92" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="H92" s="2" t="s">
-        <v>449</v>
+        <v>445</v>
       </c>
       <c r="I92" t="s">
         <v>16</v>
       </c>
       <c r="J92" s="3" t="s">
-        <v>450</v>
+        <v>446</v>
       </c>
       <c r="K92" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L92" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="93" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A93" s="11">
         <v>91</v>
       </c>
       <c r="B93">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D93" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>419</v>
-      </c>
-      <c r="F93" t="s">
-        <v>451</v>
+        <v>443</v>
+      </c>
+      <c r="F93" s="10" t="s">
+        <v>447</v>
       </c>
       <c r="G93" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="H93" s="2" t="s">
-        <v>452</v>
+        <v>448</v>
       </c>
       <c r="I93" t="s">
         <v>16</v>
       </c>
       <c r="J93" s="3" t="s">
-        <v>453</v>
+        <v>449</v>
       </c>
       <c r="K93" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L93" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="M93" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="94" spans="1:13" x14ac:dyDescent="0.2">
+    </row>
+    <row r="94" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A94" s="11">
         <v>92</v>
       </c>
       <c r="B94">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D94" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="F94" t="s">
-        <v>454</v>
+        <v>450</v>
       </c>
       <c r="G94" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="H94" s="2" t="s">
-        <v>455</v>
+        <v>451</v>
       </c>
       <c r="I94" t="s">
         <v>16</v>
       </c>
       <c r="J94" s="3" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
       <c r="K94" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L94" s="1" t="s">
         <v>19</v>
       </c>
       <c r="M94" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="95" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="J95" s="3"/>
-    </row>
-    <row r="96" spans="1:13" x14ac:dyDescent="0.2">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="95" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A95" s="11">
+        <v>93</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="D95" t="s">
+        <v>474</v>
+      </c>
+      <c r="E95" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="F95" t="s">
+        <v>453</v>
+      </c>
+      <c r="G95" t="s">
+        <v>215</v>
+      </c>
+      <c r="H95" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="I95" t="s">
+        <v>16</v>
+      </c>
+      <c r="J95" s="3" t="s">
+        <v>455</v>
+      </c>
+      <c r="K95" t="s">
+        <v>161</v>
+      </c>
+      <c r="L95" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="M95" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="96" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J96" s="3"/>
     </row>
-    <row r="97" spans="10:10" x14ac:dyDescent="0.2">
+    <row r="97" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J97" s="3"/>
     </row>
-    <row r="98" spans="10:10" x14ac:dyDescent="0.2">
+    <row r="98" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J98" s="3"/>
     </row>
-    <row r="99" spans="10:10" x14ac:dyDescent="0.2">
+    <row r="99" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J99" s="3"/>
     </row>
-    <row r="100" spans="10:10" x14ac:dyDescent="0.2">
+    <row r="100" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J100" s="3"/>
     </row>
-    <row r="101" spans="10:10" x14ac:dyDescent="0.2">
+    <row r="101" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J101" s="3"/>
+    </row>
+    <row r="102" spans="10:10" x14ac:dyDescent="0.25">
+      <c r="J102" s="3"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -5083,76 +5107,77 @@
     <hyperlink ref="J19" r:id="rId12" xr:uid="{86F5BA6B-2F60-7D4E-8748-CAE45025CAFD}"/>
     <hyperlink ref="J21" r:id="rId13" xr:uid="{BB628FDC-6C19-104A-9AB5-3CBC4E74965C}"/>
     <hyperlink ref="J22" r:id="rId14" xr:uid="{E7B042CB-521C-9A43-8413-088DADA690F6}"/>
-    <hyperlink ref="J23" r:id="rId15" xr:uid="{B354B703-65B5-1340-83BD-CCC7ACD24193}"/>
-    <hyperlink ref="J24" r:id="rId16" xr:uid="{B7B7D7AE-0E48-BD47-A53E-CA2121372461}"/>
-    <hyperlink ref="J32" r:id="rId17" xr:uid="{9C6EA54E-976E-C547-A4F6-B95CDD70C5CC}"/>
-    <hyperlink ref="J39" r:id="rId18" xr:uid="{3A8A4BF1-8B38-3547-BA26-B7CF4D96E777}"/>
-    <hyperlink ref="J54" r:id="rId19" xr:uid="{0877952C-4A88-3D48-A368-B38F86E94626}"/>
-    <hyperlink ref="J53" r:id="rId20" xr:uid="{F7F86453-3A2F-BA4B-8411-79550A1910C3}"/>
-    <hyperlink ref="J44" r:id="rId21" xr:uid="{95193995-204E-C646-AAC6-212B3970F138}"/>
-    <hyperlink ref="J37" r:id="rId22" xr:uid="{61E419F2-FA97-D342-8272-F84AAF2D1CE5}"/>
-    <hyperlink ref="J55" r:id="rId23" xr:uid="{9BF8DA02-398D-824A-9EE1-D4C13EA31FC8}"/>
-    <hyperlink ref="J45" r:id="rId24" xr:uid="{82701FD3-D585-3E41-8F88-0E90E8EE2CD7}"/>
-    <hyperlink ref="J50" r:id="rId25" xr:uid="{B3B905B2-C74E-E84F-A00B-1C1269675461}"/>
-    <hyperlink ref="J40" r:id="rId26" xr:uid="{3935EC0B-F200-C84B-84B0-F57D147181E5}"/>
-    <hyperlink ref="J41" r:id="rId27" xr:uid="{5243009C-6C68-2540-941D-394D81AD2550}"/>
-    <hyperlink ref="J43" r:id="rId28" xr:uid="{FD3E7D42-E015-E24E-8DFF-486B11773B9F}"/>
-    <hyperlink ref="J46" r:id="rId29" xr:uid="{79030505-D916-9F49-A2E5-8A35263FCB99}"/>
-    <hyperlink ref="J36" r:id="rId30" xr:uid="{F37F7670-B383-7943-8359-377911792A67}"/>
-    <hyperlink ref="J51" r:id="rId31" xr:uid="{BF64644E-9D8C-4640-BA07-CCE7AC3AF734}"/>
-    <hyperlink ref="J42" r:id="rId32" xr:uid="{C30D2353-C90E-024C-8DA8-4AC8269667EE}"/>
-    <hyperlink ref="J57" r:id="rId33" xr:uid="{77200905-4B2E-2945-AFF3-984856A66D1E}"/>
-    <hyperlink ref="J58" r:id="rId34" xr:uid="{B9EBE303-C086-9845-92F6-D928454BFF87}"/>
-    <hyperlink ref="J59" r:id="rId35" xr:uid="{876A3EAE-6E0D-7E4C-948A-B76DC12A9227}"/>
-    <hyperlink ref="J60" r:id="rId36" xr:uid="{6CBBBCB1-EBA7-E947-B5C7-008D87389A8D}"/>
-    <hyperlink ref="J61" r:id="rId37" xr:uid="{4E885EE3-55EE-CA4B-9604-C1048E2AFD1E}"/>
-    <hyperlink ref="J68" r:id="rId38" xr:uid="{DFF22E04-505B-064D-9C02-C1FB3254EFAF}"/>
-    <hyperlink ref="J62" r:id="rId39" xr:uid="{B8910815-293B-C54E-AF53-9C3A47D5D87D}"/>
-    <hyperlink ref="J64" r:id="rId40" xr:uid="{70E697E8-74B0-C349-B568-C63B64FA0418}"/>
-    <hyperlink ref="J66" r:id="rId41" xr:uid="{704F4B6C-0A8A-A844-BA76-F4B796F70244}"/>
-    <hyperlink ref="J67" r:id="rId42" xr:uid="{BEE71CB5-5764-4646-962E-C8F88260469B}"/>
-    <hyperlink ref="J69" r:id="rId43" xr:uid="{2E5CD59A-CAB7-4746-9175-BCEB0CBDADFE}"/>
-    <hyperlink ref="J70" r:id="rId44" xr:uid="{0B34B1AF-9F15-D049-91BB-5BCDCED7DD17}"/>
-    <hyperlink ref="J71" r:id="rId45" xr:uid="{A5FBDB64-8AC9-8249-AF49-952DEEC9C1C3}"/>
-    <hyperlink ref="J75" r:id="rId46" xr:uid="{34C89213-D636-8542-A477-EFFC03F657FF}"/>
-    <hyperlink ref="J73" r:id="rId47" xr:uid="{2145CC2E-D8D5-4E4A-8784-CB6349055F15}"/>
-    <hyperlink ref="J74" r:id="rId48" xr:uid="{55223226-4854-0140-A85E-AF07472C55B2}"/>
-    <hyperlink ref="J72" r:id="rId49" xr:uid="{809F7539-662F-5441-BD7A-0174489A13BB}"/>
-    <hyperlink ref="J79" r:id="rId50" xr:uid="{C5279240-4C2F-DD43-A80C-B874FE43DBD9}"/>
-    <hyperlink ref="J76" r:id="rId51" xr:uid="{A0F1EF40-FD64-8F4C-901D-2C7D1C694B61}"/>
-    <hyperlink ref="J78" r:id="rId52" xr:uid="{D71301BA-7D7E-CA49-8C1D-2A891CC213EC}"/>
+    <hyperlink ref="J24" r:id="rId15" xr:uid="{B354B703-65B5-1340-83BD-CCC7ACD24193}"/>
+    <hyperlink ref="J25" r:id="rId16" xr:uid="{B7B7D7AE-0E48-BD47-A53E-CA2121372461}"/>
+    <hyperlink ref="J33" r:id="rId17" xr:uid="{9C6EA54E-976E-C547-A4F6-B95CDD70C5CC}"/>
+    <hyperlink ref="J40" r:id="rId18" xr:uid="{3A8A4BF1-8B38-3547-BA26-B7CF4D96E777}"/>
+    <hyperlink ref="J55" r:id="rId19" xr:uid="{0877952C-4A88-3D48-A368-B38F86E94626}"/>
+    <hyperlink ref="J54" r:id="rId20" xr:uid="{F7F86453-3A2F-BA4B-8411-79550A1910C3}"/>
+    <hyperlink ref="J45" r:id="rId21" xr:uid="{95193995-204E-C646-AAC6-212B3970F138}"/>
+    <hyperlink ref="J38" r:id="rId22" xr:uid="{61E419F2-FA97-D342-8272-F84AAF2D1CE5}"/>
+    <hyperlink ref="J56" r:id="rId23" xr:uid="{9BF8DA02-398D-824A-9EE1-D4C13EA31FC8}"/>
+    <hyperlink ref="J46" r:id="rId24" xr:uid="{82701FD3-D585-3E41-8F88-0E90E8EE2CD7}"/>
+    <hyperlink ref="J51" r:id="rId25" xr:uid="{B3B905B2-C74E-E84F-A00B-1C1269675461}"/>
+    <hyperlink ref="J41" r:id="rId26" xr:uid="{3935EC0B-F200-C84B-84B0-F57D147181E5}"/>
+    <hyperlink ref="J42" r:id="rId27" xr:uid="{5243009C-6C68-2540-941D-394D81AD2550}"/>
+    <hyperlink ref="J44" r:id="rId28" xr:uid="{FD3E7D42-E015-E24E-8DFF-486B11773B9F}"/>
+    <hyperlink ref="J47" r:id="rId29" xr:uid="{79030505-D916-9F49-A2E5-8A35263FCB99}"/>
+    <hyperlink ref="J37" r:id="rId30" xr:uid="{F37F7670-B383-7943-8359-377911792A67}"/>
+    <hyperlink ref="J52" r:id="rId31" xr:uid="{BF64644E-9D8C-4640-BA07-CCE7AC3AF734}"/>
+    <hyperlink ref="J43" r:id="rId32" xr:uid="{C30D2353-C90E-024C-8DA8-4AC8269667EE}"/>
+    <hyperlink ref="J58" r:id="rId33" xr:uid="{77200905-4B2E-2945-AFF3-984856A66D1E}"/>
+    <hyperlink ref="J59" r:id="rId34" xr:uid="{B9EBE303-C086-9845-92F6-D928454BFF87}"/>
+    <hyperlink ref="J60" r:id="rId35" xr:uid="{876A3EAE-6E0D-7E4C-948A-B76DC12A9227}"/>
+    <hyperlink ref="J61" r:id="rId36" xr:uid="{6CBBBCB1-EBA7-E947-B5C7-008D87389A8D}"/>
+    <hyperlink ref="J62" r:id="rId37" xr:uid="{4E885EE3-55EE-CA4B-9604-C1048E2AFD1E}"/>
+    <hyperlink ref="J69" r:id="rId38" xr:uid="{DFF22E04-505B-064D-9C02-C1FB3254EFAF}"/>
+    <hyperlink ref="J63" r:id="rId39" xr:uid="{B8910815-293B-C54E-AF53-9C3A47D5D87D}"/>
+    <hyperlink ref="J65" r:id="rId40" xr:uid="{70E697E8-74B0-C349-B568-C63B64FA0418}"/>
+    <hyperlink ref="J67" r:id="rId41" xr:uid="{704F4B6C-0A8A-A844-BA76-F4B796F70244}"/>
+    <hyperlink ref="J68" r:id="rId42" xr:uid="{BEE71CB5-5764-4646-962E-C8F88260469B}"/>
+    <hyperlink ref="J70" r:id="rId43" xr:uid="{2E5CD59A-CAB7-4746-9175-BCEB0CBDADFE}"/>
+    <hyperlink ref="J71" r:id="rId44" xr:uid="{0B34B1AF-9F15-D049-91BB-5BCDCED7DD17}"/>
+    <hyperlink ref="J72" r:id="rId45" xr:uid="{A5FBDB64-8AC9-8249-AF49-952DEEC9C1C3}"/>
+    <hyperlink ref="J76" r:id="rId46" xr:uid="{34C89213-D636-8542-A477-EFFC03F657FF}"/>
+    <hyperlink ref="J74" r:id="rId47" xr:uid="{2145CC2E-D8D5-4E4A-8784-CB6349055F15}"/>
+    <hyperlink ref="J75" r:id="rId48" xr:uid="{55223226-4854-0140-A85E-AF07472C55B2}"/>
+    <hyperlink ref="J73" r:id="rId49" xr:uid="{809F7539-662F-5441-BD7A-0174489A13BB}"/>
+    <hyperlink ref="J80" r:id="rId50" xr:uid="{C5279240-4C2F-DD43-A80C-B874FE43DBD9}"/>
+    <hyperlink ref="J77" r:id="rId51" xr:uid="{A0F1EF40-FD64-8F4C-901D-2C7D1C694B61}"/>
+    <hyperlink ref="J79" r:id="rId52" xr:uid="{D71301BA-7D7E-CA49-8C1D-2A891CC213EC}"/>
     <hyperlink ref="J6" r:id="rId53" xr:uid="{76D0266E-10CB-E142-860A-795E931F7524}"/>
     <hyperlink ref="J18" r:id="rId54" xr:uid="{BD3BE890-A95E-0E44-B620-11E20304C92F}"/>
     <hyperlink ref="J20" r:id="rId55" xr:uid="{D3E510DF-6DCE-8C44-A6BA-A0DDF9CFB434}"/>
-    <hyperlink ref="J56" r:id="rId56" xr:uid="{8E140BB9-7AFC-604A-8B3D-1B04CD5E5F89}"/>
-    <hyperlink ref="J47" r:id="rId57" xr:uid="{9D94EED0-848B-A948-879C-46720FD3C7DF}"/>
-    <hyperlink ref="J48" r:id="rId58" xr:uid="{3279F53D-E307-774B-8B0F-95F4175CC0DE}"/>
-    <hyperlink ref="J81" r:id="rId59" xr:uid="{B011BC21-C74A-C94D-B085-A2AFD8A426A7}"/>
-    <hyperlink ref="J82" r:id="rId60" xr:uid="{B057E7E7-8B8C-704D-92C7-FF0E276E14BB}"/>
-    <hyperlink ref="J80" r:id="rId61" xr:uid="{AA2427B9-63E3-1E49-B38C-45CCDBD46A41}"/>
-    <hyperlink ref="J83" r:id="rId62" xr:uid="{C8AA8233-DAE5-5F41-941D-130E77D7237B}"/>
-    <hyperlink ref="J88" r:id="rId63" xr:uid="{F97C1FC4-DEA3-D047-8574-6EA3EC99CDD5}"/>
-    <hyperlink ref="J90" r:id="rId64" xr:uid="{DB61E21C-9988-424F-8BF3-2AF8B50ADC77}"/>
-    <hyperlink ref="J85" r:id="rId65" xr:uid="{0746EBE0-5668-854E-B70D-4883B693EB08}"/>
-    <hyperlink ref="J84" r:id="rId66" xr:uid="{AE9AA9CC-3F25-BA4A-A596-3A43094BABF1}"/>
-    <hyperlink ref="J25" r:id="rId67" xr:uid="{B5D12788-30BC-F34D-8EA9-80C31BB0DBD0}"/>
-    <hyperlink ref="J27" r:id="rId68" xr:uid="{0EB2898D-DE96-BA47-BD8D-28F7DDFA6E2A}"/>
-    <hyperlink ref="J28" r:id="rId69" xr:uid="{9B7DB72F-D84A-BB47-A90F-DAAA9233E2FE}"/>
-    <hyperlink ref="J52" r:id="rId70" xr:uid="{8FB0D08D-C1DE-F64B-B871-AF85B39521D2}"/>
-    <hyperlink ref="J89" r:id="rId71" xr:uid="{B963E2A1-1BD1-7D46-A4F7-FB6638223298}"/>
-    <hyperlink ref="J65" r:id="rId72" xr:uid="{202ECC15-B5F1-194D-B748-16115594F03F}"/>
-    <hyperlink ref="J92" r:id="rId73" xr:uid="{CB201C2D-6C7A-2642-9579-7C00E5FABD60}"/>
-    <hyperlink ref="J91" r:id="rId74" xr:uid="{62446F2D-7CDA-F64E-B35D-D983A5F17F8C}"/>
+    <hyperlink ref="J57" r:id="rId56" xr:uid="{8E140BB9-7AFC-604A-8B3D-1B04CD5E5F89}"/>
+    <hyperlink ref="J48" r:id="rId57" xr:uid="{9D94EED0-848B-A948-879C-46720FD3C7DF}"/>
+    <hyperlink ref="J49" r:id="rId58" xr:uid="{3279F53D-E307-774B-8B0F-95F4175CC0DE}"/>
+    <hyperlink ref="J82" r:id="rId59" xr:uid="{B011BC21-C74A-C94D-B085-A2AFD8A426A7}"/>
+    <hyperlink ref="J83" r:id="rId60" xr:uid="{B057E7E7-8B8C-704D-92C7-FF0E276E14BB}"/>
+    <hyperlink ref="J81" r:id="rId61" xr:uid="{AA2427B9-63E3-1E49-B38C-45CCDBD46A41}"/>
+    <hyperlink ref="J84" r:id="rId62" xr:uid="{C8AA8233-DAE5-5F41-941D-130E77D7237B}"/>
+    <hyperlink ref="J89" r:id="rId63" xr:uid="{F97C1FC4-DEA3-D047-8574-6EA3EC99CDD5}"/>
+    <hyperlink ref="J91" r:id="rId64" xr:uid="{DB61E21C-9988-424F-8BF3-2AF8B50ADC77}"/>
+    <hyperlink ref="J86" r:id="rId65" xr:uid="{0746EBE0-5668-854E-B70D-4883B693EB08}"/>
+    <hyperlink ref="J85" r:id="rId66" xr:uid="{AE9AA9CC-3F25-BA4A-A596-3A43094BABF1}"/>
+    <hyperlink ref="J26" r:id="rId67" xr:uid="{B5D12788-30BC-F34D-8EA9-80C31BB0DBD0}"/>
+    <hyperlink ref="J28" r:id="rId68" xr:uid="{0EB2898D-DE96-BA47-BD8D-28F7DDFA6E2A}"/>
+    <hyperlink ref="J29" r:id="rId69" xr:uid="{9B7DB72F-D84A-BB47-A90F-DAAA9233E2FE}"/>
+    <hyperlink ref="J53" r:id="rId70" xr:uid="{8FB0D08D-C1DE-F64B-B871-AF85B39521D2}"/>
+    <hyperlink ref="J90" r:id="rId71" xr:uid="{B963E2A1-1BD1-7D46-A4F7-FB6638223298}"/>
+    <hyperlink ref="J66" r:id="rId72" xr:uid="{202ECC15-B5F1-194D-B748-16115594F03F}"/>
+    <hyperlink ref="J93" r:id="rId73" xr:uid="{CB201C2D-6C7A-2642-9579-7C00E5FABD60}"/>
+    <hyperlink ref="J92" r:id="rId74" xr:uid="{62446F2D-7CDA-F64E-B35D-D983A5F17F8C}"/>
     <hyperlink ref="J10" r:id="rId75" xr:uid="{2509C66A-91EC-9440-B040-702A9DF1869B}"/>
     <hyperlink ref="J11" r:id="rId76" xr:uid="{BE6DF33C-7BD8-804B-8DD3-29A0A3CAE976}"/>
-    <hyperlink ref="J49" r:id="rId77" xr:uid="{4F9959A3-DA08-A548-9E07-32CD80A8EFB9}"/>
-    <hyperlink ref="J63" r:id="rId78" xr:uid="{953EB46E-B69E-D846-9342-707BB3B28D22}"/>
-    <hyperlink ref="J77" r:id="rId79" xr:uid="{44D53F63-A76D-9146-96CD-8719FEE5385E}"/>
-    <hyperlink ref="J93" r:id="rId80" xr:uid="{3C66832E-3AAC-BD4C-B893-229986E5416C}"/>
-    <hyperlink ref="J94" r:id="rId81" xr:uid="{5E833CF6-CEF8-7C43-8234-9528E6420F9C}"/>
-    <hyperlink ref="J87" r:id="rId82" xr:uid="{7A3102F2-2618-4F40-9A02-057AD103DA8E}"/>
-    <hyperlink ref="J86" r:id="rId83" xr:uid="{310A59EB-D532-0B45-B24F-100BB497BF4C}"/>
-    <hyperlink ref="J30" r:id="rId84" xr:uid="{A7659882-810F-224A-8835-DB9C6A77F501}"/>
+    <hyperlink ref="J50" r:id="rId77" xr:uid="{4F9959A3-DA08-A548-9E07-32CD80A8EFB9}"/>
+    <hyperlink ref="J64" r:id="rId78" xr:uid="{953EB46E-B69E-D846-9342-707BB3B28D22}"/>
+    <hyperlink ref="J78" r:id="rId79" xr:uid="{44D53F63-A76D-9146-96CD-8719FEE5385E}"/>
+    <hyperlink ref="J94" r:id="rId80" xr:uid="{3C66832E-3AAC-BD4C-B893-229986E5416C}"/>
+    <hyperlink ref="J95" r:id="rId81" xr:uid="{5E833CF6-CEF8-7C43-8234-9528E6420F9C}"/>
+    <hyperlink ref="J88" r:id="rId82" xr:uid="{7A3102F2-2618-4F40-9A02-057AD103DA8E}"/>
+    <hyperlink ref="J87" r:id="rId83" xr:uid="{310A59EB-D532-0B45-B24F-100BB497BF4C}"/>
+    <hyperlink ref="J31" r:id="rId84" xr:uid="{A7659882-810F-224A-8835-DB9C6A77F501}"/>
+    <hyperlink ref="J23" r:id="rId85" display="490-1451-1-ND" xr:uid="{C84A6422-C4D0-4017-B3BB-8DF7D90E28A8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>